<commit_message>
COMITY: final da aula
</commit_message>
<xml_diff>
--- a/Plano_de_teste.xlsx
+++ b/Plano_de_teste.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\Escola\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\SENAI\Desktop\teste-de-software-1S2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F0A87F8E-C184-4425-9DD8-F2922A06C085}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C2AF8F2-E762-4DD7-AA4E-0623451A8096}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" xr2:uid="{DFF2E1B7-49BA-47E2-A8F8-B0B6A55874AE}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12225" activeTab="1" xr2:uid="{DFF2E1B7-49BA-47E2-A8F8-B0B6A55874AE}"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="Planilha1 (2)" sheetId="4" r:id="rId1"/>
+    <sheet name="Planilha1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="168" uniqueCount="66">
   <si>
     <t>TIPO DE TESTE</t>
   </si>
@@ -115,6 +116,114 @@
   </si>
   <si>
     <t>Verificando um número maior que 10</t>
+  </si>
+  <si>
+    <t>boletim.calculos</t>
+  </si>
+  <si>
+    <t>calcular_media</t>
+  </si>
+  <si>
+    <t>UNITÁRIO</t>
+  </si>
+  <si>
+    <t>Teste com notas inteiras</t>
+  </si>
+  <si>
+    <t>[8, 10]</t>
+  </si>
+  <si>
+    <t>9.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNITÁRIO </t>
+  </si>
+  <si>
+    <t>Teste com notas quebradas</t>
+  </si>
+  <si>
+    <t>[9.5, 4.7]</t>
+  </si>
+  <si>
+    <t>7.1</t>
+  </si>
+  <si>
+    <t>Se por string como entrada</t>
+  </si>
+  <si>
+    <t>typeError:"entrada invalida"</t>
+  </si>
+  <si>
+    <t>Se por numero negativo</t>
+  </si>
+  <si>
+    <t>valueError:"entrada invalida"</t>
+  </si>
+  <si>
+    <t>Se por numero maior que 10</t>
+  </si>
+  <si>
+    <t>["DOIS", "TRES"]</t>
+  </si>
+  <si>
+    <t>[-5, -4 ]</t>
+  </si>
+  <si>
+    <t>[15, 20]</t>
+  </si>
+  <si>
+    <t>Teste com muitas notas</t>
+  </si>
+  <si>
+    <t>[9, 10, 10, 5.5, 8, 9, 5.4]</t>
+  </si>
+  <si>
+    <t>Se por os numeros sem uma lista</t>
+  </si>
+  <si>
+    <t>10, 4</t>
+  </si>
+  <si>
+    <t>Teste co apenas um numero</t>
+  </si>
+  <si>
+    <t>[5]</t>
+  </si>
+  <si>
+    <t>Teste apenas com notas 10</t>
+  </si>
+  <si>
+    <t>[10, 10, 10]</t>
+  </si>
+  <si>
+    <t>Teste com notas decimais e inteiras</t>
+  </si>
+  <si>
+    <t>[10, 7.5, 9, 9.5]</t>
+  </si>
+  <si>
+    <t>5.0</t>
+  </si>
+  <si>
+    <t>8.12</t>
+  </si>
+  <si>
+    <t>10.0</t>
+  </si>
+  <si>
+    <t>Teste apenas com notas 0</t>
+  </si>
+  <si>
+    <t>[0, 0, 0]</t>
+  </si>
+  <si>
+    <t>0.0</t>
+  </si>
+  <si>
+    <t>Se entregar a lista vazia</t>
+  </si>
+  <si>
+    <t>[ ]</t>
   </si>
 </sst>
 </file>
@@ -207,54 +316,23 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="18">
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="4" tint="-0.249977111117893"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="36">
     <dxf>
       <font>
         <b val="0"/>
@@ -334,25 +412,164 @@
       <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <bottom style="thin">
+          <color rgb="FF4472C4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color rgb="FF4472C4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -362,11 +579,47 @@
       </border>
     </dxf>
     <dxf>
-      <border outline="0">
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-      </border>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="4" tint="-0.249977111117893"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -388,33 +641,66 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{70E3F201-B8AD-4A2C-B1D2-80F380021684}" name="Tabela3" displayName="Tabela3" ref="A3:F12" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{9E62F754-97D9-40D7-9141-E211B7F89CA1}" name="Tabela32" displayName="Tabela32" ref="A3:F12" totalsRowShown="0" headerRowDxfId="20" dataDxfId="19">
   <autoFilter ref="A3:F12" xr:uid="{6467301A-9E73-4F44-BEEF-C1E28452C844}"/>
   <sortState ref="A4:F10">
     <sortCondition ref="F3:F10"/>
   </sortState>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{D2617CB4-56D7-4510-804E-B66A17324D75}" name="TIPO DE TESTE" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{F71473C1-80FC-475A-AB10-1DCE874C027B}" name="ARQUIVOS" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{2F1E1CF9-E654-47DF-AE7B-ABB4531DA66F}" name="FUNÇÕES" dataDxfId="13"/>
-    <tableColumn id="4" xr3:uid="{3EBEE7BB-A771-423C-BD7A-5FEB8C7C511F}" name="TESTE" dataDxfId="12"/>
-    <tableColumn id="5" xr3:uid="{C1A88667-A341-4D13-B119-84315C30D4EC}" name="ENTRADA" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{46112BEF-7B28-4018-8F34-412DAEA12C41}" name="SAIDA" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{7DC98F05-DE72-461E-8A8A-F357DEF09A9C}" name="TIPO DE TESTE" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{80598200-B41F-4453-B286-CFAA8E3BEB61}" name="ARQUIVOS" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{FF65E73C-C1C1-49A5-B768-65BFE5B4068B}" name="FUNÇÕES" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{5B5967A6-C7C3-4FA7-A2BA-9B9ECE48D5C2}" name="TESTE" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{C40E938D-CA9E-4AAF-AAC4-54DBA648C001}" name="ENTRADA" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{B53FCCAC-FEF4-44B2-9B25-74E926CCE47E}" name="SAIDA" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{60435578-CBCB-44E2-9FB4-9AAA09DDDDF2}" name="Tabela6" displayName="Tabela6" ref="A16:F19" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowBorderDxfId="16" tableBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{27F6F75F-1021-47F3-8ADA-137FD074E215}" name="Tabela63" displayName="Tabela63" ref="A16:F19" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11" headerRowBorderDxfId="9" tableBorderDxfId="10">
   <autoFilter ref="A16:F19" xr:uid="{3A388368-B54B-4430-963C-2A256FC153F3}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{3F6CFDB9-2737-4DBA-A536-B2C143F50F2F}" name="TIPO DE TESTE" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{67F70CD4-ACB9-44FF-9770-C0906FD1DA59}" name="ARQUIVOS" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{205A854C-D308-44D9-9D40-D69A8C27E624}" name="FUNÇÕES" dataDxfId="5"/>
-    <tableColumn id="4" xr3:uid="{085BE3A5-476A-40D8-8D82-3B5DB41CC09F}" name="TESTE" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{3DFBB1B0-D2FC-4274-86E9-665AB4B7B387}" name="ENTRADA" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{9704FEBE-5E9C-40FC-A21F-4F8930415098}" name="SAIDA" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{4E1F7F9A-FC81-4535-93BC-E7135C9B8B19}" name="TIPO DE TESTE" dataDxfId="8"/>
+    <tableColumn id="2" xr3:uid="{700B5C41-267A-492B-85F8-A64BEA2E143E}" name="ARQUIVOS" dataDxfId="7"/>
+    <tableColumn id="3" xr3:uid="{81EC6BC2-42DE-4DDF-A241-DDF306684DEF}" name="FUNÇÕES" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{3A581C0C-B578-4B1D-959E-A121AD4D78CA}" name="TESTE" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{82029259-76A0-4C77-80F1-7608B4F19E35}" name="ENTRADA" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{9F84F326-6D79-482D-A0D3-5138FE04B705}" name="SAIDA" dataDxfId="3"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{70E3F201-B8AD-4A2C-B1D2-80F380021684}" name="Tabela3" displayName="Tabela3" ref="A3:F12" totalsRowShown="0" headerRowDxfId="35" dataDxfId="34">
+  <autoFilter ref="A3:F12" xr:uid="{6467301A-9E73-4F44-BEEF-C1E28452C844}"/>
+  <sortState ref="A4:F10">
+    <sortCondition ref="F3:F10"/>
+  </sortState>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{D2617CB4-56D7-4510-804E-B66A17324D75}" name="TIPO DE TESTE" dataDxfId="33"/>
+    <tableColumn id="2" xr3:uid="{F71473C1-80FC-475A-AB10-1DCE874C027B}" name="ARQUIVOS" dataDxfId="32"/>
+    <tableColumn id="3" xr3:uid="{2F1E1CF9-E654-47DF-AE7B-ABB4531DA66F}" name="FUNÇÕES" dataDxfId="31"/>
+    <tableColumn id="4" xr3:uid="{3EBEE7BB-A771-423C-BD7A-5FEB8C7C511F}" name="TESTE" dataDxfId="30"/>
+    <tableColumn id="5" xr3:uid="{C1A88667-A341-4D13-B119-84315C30D4EC}" name="ENTRADA" dataDxfId="29"/>
+    <tableColumn id="6" xr3:uid="{46112BEF-7B28-4018-8F34-412DAEA12C41}" name="SAIDA" dataDxfId="28"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{60435578-CBCB-44E2-9FB4-9AAA09DDDDF2}" name="Tabela6" displayName="Tabela6" ref="A16:F21" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24">
+  <autoFilter ref="A16:F21" xr:uid="{3A388368-B54B-4430-963C-2A256FC153F3}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{3F6CFDB9-2737-4DBA-A536-B2C143F50F2F}" name="TIPO DE TESTE" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{67F70CD4-ACB9-44FF-9770-C0906FD1DA59}" name="ARQUIVOS" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{205A854C-D308-44D9-9D40-D69A8C27E624}" name="FUNÇÕES" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{085BE3A5-476A-40D8-8D82-3B5DB41CC09F}" name="TESTE" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{3DFBB1B0-D2FC-4274-86E9-665AB4B7B387}" name="ENTRADA" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{9704FEBE-5E9C-40FC-A21F-4F8930415098}" name="SAIDA" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -716,7 +1002,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ECF97B2-6F2A-40BC-B329-781313933B0E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7258330E-A74B-4F1A-93DB-1AD22A3E5794}">
   <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -728,22 +1014,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3"/>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -954,40 +1240,40 @@
       <c r="F13" s="1"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="5"/>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="4" t="s">
+      <c r="A16" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B16" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="C16" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D16" s="4" t="s">
+      <c r="D16" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E16" s="4" t="s">
+      <c r="E16" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F16" s="4" t="s">
+      <c r="F16" s="3" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1049,6 +1335,384 @@
       </c>
       <c r="F19" s="1" t="s">
         <v>28</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F2"/>
+    <mergeCell ref="A14:F15"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <tableParts count="2">
+    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0ECF97B2-6F2A-40BC-B329-781313933B0E}">
+  <dimension ref="A1:F21"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="48" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D11" s="1"/>
+      <c r="E11" s="1"/>
+      <c r="F11" s="1"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="1"/>
+      <c r="E12" s="1"/>
+      <c r="F12" s="1"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="1"/>
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="1"/>
+      <c r="E13" s="1"/>
+      <c r="F13" s="1"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>